<commit_message>
pagination code is changed
</commit_message>
<xml_diff>
--- a/tests/Employee/downloads/exported_employees.xlsx
+++ b/tests/Employee/downloads/exported_employees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J54"/>
+  <dimension ref="A1:J55"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -433,28 +433,28 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>BITECOS1373</v>
+        <v>BITECOS1374</v>
       </c>
       <c r="B2" t="str">
-        <v>boopati</v>
+        <v>EditTest_41521</v>
       </c>
       <c r="C2" t="str">
-        <v>boopati@yopmail.com</v>
+        <v>chandrika_40975@yopmail.com</v>
       </c>
       <c r="D2" t="str">
-        <v>2026-07-15</v>
+        <v>2026-07-14</v>
       </c>
       <c r="E2" t="str">
-        <v>Logistics</v>
+        <v>Finance</v>
       </c>
       <c r="F2" t="str">
-        <v>Warehouse Specialist</v>
+        <v>Finance Manager</v>
       </c>
       <c r="G2" t="str">
-        <v>VijayKumar S Kale</v>
+        <v>Kavya TN</v>
       </c>
       <c r="H2" t="str">
-        <v>Tumkur</v>
+        <v>Bangalore</v>
       </c>
       <c r="I2" t="str">
         <v>Active</v>
@@ -465,28 +465,28 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>BITECOS1372</v>
+        <v>BITECOS1373</v>
       </c>
       <c r="B3" t="str">
-        <v>Chandrika_test</v>
+        <v>boopati</v>
       </c>
       <c r="C3" t="str">
-        <v>chandrika05@yopmail.com</v>
+        <v>boopati@yopmail.com</v>
       </c>
       <c r="D3" t="str">
-        <v>2025-01-01</v>
+        <v>2026-07-15</v>
       </c>
       <c r="E3" t="str">
         <v>Logistics</v>
       </c>
       <c r="F3" t="str">
-        <v>Warehouse Supervisor</v>
+        <v>Warehouse Specialist</v>
       </c>
       <c r="G3" t="str">
-        <v>Kavya TN</v>
+        <v>VijayKumar S Kale</v>
       </c>
       <c r="H3" t="str">
-        <v xml:space="preserve">HAL Bangalore </v>
+        <v>Tumkur</v>
       </c>
       <c r="I3" t="str">
         <v>Active</v>
@@ -497,16 +497,16 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>BITECOS1371</v>
+        <v>BITECOS1372</v>
       </c>
       <c r="B4" t="str">
-        <v>chandrika_47312</v>
+        <v>Chandrika_test</v>
       </c>
       <c r="C4" t="str">
-        <v>chandrika_47312@yopmail.com</v>
+        <v>chandrika05@yopmail.com</v>
       </c>
       <c r="D4" t="str">
-        <v>2026-07-14</v>
+        <v>2025-01-01</v>
       </c>
       <c r="E4" t="str">
         <v>Logistics</v>
@@ -518,7 +518,7 @@
         <v>Kavya TN</v>
       </c>
       <c r="H4" t="str">
-        <v>Bangalore</v>
+        <v xml:space="preserve">HAL Bangalore </v>
       </c>
       <c r="I4" t="str">
         <v>Active</v>
@@ -529,13 +529,13 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>BITECOS1370</v>
+        <v>BITECOS1371</v>
       </c>
       <c r="B5" t="str">
-        <v>chandrika_65432</v>
+        <v>chandrika_47312</v>
       </c>
       <c r="C5" t="str">
-        <v>chandrika_65432@yopmail.com</v>
+        <v>chandrika_47312@yopmail.com</v>
       </c>
       <c r="D5" t="str">
         <v>2026-07-14</v>
@@ -553,7 +553,7 @@
         <v>Bangalore</v>
       </c>
       <c r="I5" t="str">
-        <v>Inactive</v>
+        <v>Active</v>
       </c>
       <c r="J5" t="str">
         <v>Yes</v>
@@ -561,22 +561,22 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>BITECOS1369</v>
+        <v>BITECOS1370</v>
       </c>
       <c r="B6" t="str">
-        <v>EditTest_56998</v>
+        <v>chandrika_65432</v>
       </c>
       <c r="C6" t="str">
-        <v>chandrika_25408@yopmail.com</v>
+        <v>chandrika_65432@yopmail.com</v>
       </c>
       <c r="D6" t="str">
         <v>2026-07-14</v>
       </c>
       <c r="E6" t="str">
-        <v>Finance</v>
+        <v>Logistics</v>
       </c>
       <c r="F6" t="str">
-        <v>Finance Manager</v>
+        <v>Warehouse Supervisor</v>
       </c>
       <c r="G6" t="str">
         <v>Kavya TN</v>
@@ -588,65 +588,65 @@
         <v>Active</v>
       </c>
       <c r="J6" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>BITECOS1368</v>
+        <v>BITECOS1369</v>
       </c>
       <c r="B7" t="str">
-        <v>edited_name_x72h5</v>
+        <v>EditTest_56998</v>
       </c>
       <c r="C7" t="str">
-        <v>chandrika_yspcp@yopmail.com</v>
+        <v>chandrika_25408@yopmail.com</v>
       </c>
       <c r="D7" t="str">
-        <v>2026-07-15</v>
+        <v>2026-07-14</v>
       </c>
       <c r="E7" t="str">
-        <v>Services</v>
+        <v>Finance</v>
       </c>
       <c r="F7" t="str">
-        <v>Warehouse Supervisor</v>
+        <v>Finance Manager</v>
       </c>
       <c r="G7" t="str">
-        <v>Ramesh Mali</v>
+        <v>Kavya TN</v>
       </c>
       <c r="H7" t="str">
-        <v>626637367464</v>
+        <v>Bangalore</v>
       </c>
       <c r="I7" t="str">
-        <v>Active</v>
+        <v>Inactive</v>
       </c>
       <c r="J7" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>BITECOS1367</v>
+        <v>BITECOS1368</v>
       </c>
       <c r="B8" t="str">
-        <v>edited_name_67gum</v>
+        <v>edited_name_x72h5</v>
       </c>
       <c r="C8" t="str">
-        <v>edited_name_a4id6@yopmail.com</v>
+        <v>chandrika_yspcp@yopmail.com</v>
       </c>
       <c r="D8" t="str">
-        <v>2026-07-16</v>
+        <v>2026-07-15</v>
       </c>
       <c r="E8" t="str">
-        <v>Shipment</v>
+        <v>Services</v>
       </c>
       <c r="F8" t="str">
         <v>Warehouse Supervisor</v>
       </c>
       <c r="G8" t="str">
-        <v>Devakumar N</v>
+        <v>Ramesh Mali</v>
       </c>
       <c r="H8" t="str">
-        <v>Coimbatore</v>
+        <v>626637367464</v>
       </c>
       <c r="I8" t="str">
         <v>Active</v>
@@ -657,28 +657,28 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>BITECOS1366</v>
+        <v>BITECOS1367</v>
       </c>
       <c r="B9" t="str">
-        <v>chandrika_vulapu</v>
+        <v>edited_name_67gum</v>
       </c>
       <c r="C9" t="str">
-        <v>chandrika01@yop.com</v>
+        <v>edited_name_a4id6@yopmail.com</v>
       </c>
       <c r="D9" t="str">
-        <v>2026-07-14</v>
+        <v>2026-07-16</v>
       </c>
       <c r="E9" t="str">
-        <v>Logistics</v>
+        <v>Shipment</v>
       </c>
       <c r="F9" t="str">
         <v>Warehouse Supervisor</v>
       </c>
       <c r="G9" t="str">
-        <v>Kavya TN</v>
+        <v>Devakumar N</v>
       </c>
       <c r="H9" t="str">
-        <v>Bangalore</v>
+        <v>Coimbatore</v>
       </c>
       <c r="I9" t="str">
         <v>Active</v>
@@ -689,13 +689,13 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>BITECOS1365</v>
+        <v>BITECOS1366</v>
       </c>
       <c r="B10" t="str">
-        <v>chandrika</v>
+        <v>chandrika_vulapu</v>
       </c>
       <c r="C10" t="str">
-        <v>chandrika@yop.com</v>
+        <v>chandrika01@yop.com</v>
       </c>
       <c r="D10" t="str">
         <v>2026-07-14</v>
@@ -713,7 +713,7 @@
         <v>Bangalore</v>
       </c>
       <c r="I10" t="str">
-        <v>Active</v>
+        <v>Inactive</v>
       </c>
       <c r="J10" t="str">
         <v>Yes</v>
@@ -721,13 +721,13 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>BITECOS1364</v>
+        <v>BITECOS1365</v>
       </c>
       <c r="B11" t="str">
-        <v>ycgeisyhjc</v>
+        <v>chandrika</v>
       </c>
       <c r="C11" t="str">
-        <v>rjbkerj@yopmail.com</v>
+        <v>chandrika@yop.com</v>
       </c>
       <c r="D11" t="str">
         <v>2026-07-14</v>
@@ -739,10 +739,10 @@
         <v>Warehouse Supervisor</v>
       </c>
       <c r="G11" t="str">
-        <v>VijayKumar S Kale</v>
+        <v>Kavya TN</v>
       </c>
       <c r="H11" t="str">
-        <v>626637367464</v>
+        <v>Bangalore</v>
       </c>
       <c r="I11" t="str">
         <v>Active</v>
@@ -753,28 +753,28 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>BITECOS1363</v>
+        <v>BITECOS1364</v>
       </c>
       <c r="B12" t="str">
-        <v>Bala Subramanya Iyyangar</v>
+        <v>ycgeisyhjc</v>
       </c>
       <c r="C12" t="str">
-        <v>Balaiyyangar3@yopmail.com</v>
+        <v>rjbkerj@yopmail.com</v>
       </c>
       <c r="D12" t="str">
-        <v>2026-06-16</v>
+        <v>2026-07-14</v>
       </c>
       <c r="E12" t="str">
-        <v>Shipment</v>
+        <v>Logistics</v>
       </c>
       <c r="F12" t="str">
-        <v>Zoho Developer</v>
+        <v>Warehouse Supervisor</v>
       </c>
       <c r="G12" t="str">
-        <v>Bandi Prasanth Babu</v>
+        <v>VijayKumar S Kale</v>
       </c>
       <c r="H12" t="str">
-        <v xml:space="preserve">HAL Bangalore </v>
+        <v>626637367464</v>
       </c>
       <c r="I12" t="str">
         <v>Active</v>
@@ -785,16 +785,16 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>BITECOS1362</v>
+        <v>BITECOS1363</v>
       </c>
       <c r="B13" t="str">
-        <v>Anish Kumar</v>
+        <v>Bala Subramanya Iyyangar</v>
       </c>
       <c r="C13" t="str">
-        <v>anish.kumar@brilyant.com</v>
+        <v>Balaiyyangar3@yopmail.com</v>
       </c>
       <c r="D13" t="str">
-        <v>2023-06-01</v>
+        <v>2026-06-16</v>
       </c>
       <c r="E13" t="str">
         <v>Shipment</v>
@@ -803,10 +803,10 @@
         <v>Zoho Developer</v>
       </c>
       <c r="G13" t="str">
-        <v>Bhanu Prakash</v>
+        <v>Bandi Prasanth Babu</v>
       </c>
       <c r="H13" t="str">
-        <v>Gurugram</v>
+        <v xml:space="preserve">HAL Bangalore </v>
       </c>
       <c r="I13" t="str">
         <v>Active</v>
@@ -817,16 +817,16 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>BITECOS1361</v>
+        <v>BITECOS1362</v>
       </c>
       <c r="B14" t="str">
-        <v>Vasanth Kumar</v>
+        <v>Anish Kumar</v>
       </c>
       <c r="C14" t="str">
-        <v>vasanthakumar.g@brilyant.com</v>
+        <v>anish.kumar@brilyant.com</v>
       </c>
       <c r="D14" t="str">
-        <v>2026-05-01</v>
+        <v>2023-06-01</v>
       </c>
       <c r="E14" t="str">
         <v>Shipment</v>
@@ -835,10 +835,10 @@
         <v>Zoho Developer</v>
       </c>
       <c r="G14" t="str">
-        <v>S Jagadesh</v>
+        <v>Bhanu Prakash</v>
       </c>
       <c r="H14" t="str">
-        <v>Kerala</v>
+        <v>Gurugram</v>
       </c>
       <c r="I14" t="str">
         <v>Active</v>
@@ -849,48 +849,48 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>BITECOS1360</v>
+        <v>BITECOS1361</v>
       </c>
       <c r="B15" t="str">
-        <v>Thomas J</v>
+        <v>Vasanth Kumar</v>
       </c>
       <c r="C15" t="str">
-        <v>zensar.demo1@brilyant.com</v>
+        <v>vasanthakumar.g@brilyant.com</v>
       </c>
       <c r="D15" t="str">
-        <v>2026-05-18</v>
+        <v>2026-05-01</v>
       </c>
       <c r="E15" t="str">
         <v>Shipment</v>
       </c>
       <c r="F15" t="str">
-        <v>Python Developer</v>
+        <v>Zoho Developer</v>
       </c>
       <c r="G15" t="str">
-        <v>Bhanu Prakash</v>
+        <v>S Jagadesh</v>
       </c>
       <c r="H15" t="str">
-        <v>Coimbatore</v>
+        <v>Kerala</v>
       </c>
       <c r="I15" t="str">
-        <v>Inactive</v>
+        <v>Active</v>
       </c>
       <c r="J15" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>BITECOS1359</v>
+        <v>BITECOS1360</v>
       </c>
       <c r="B16" t="str">
-        <v>Ravi Rhanderj</v>
+        <v>Thomas J</v>
       </c>
       <c r="C16" t="str">
-        <v>zensar.demo@brilyant.com</v>
+        <v>zensar.demo1@brilyant.com</v>
       </c>
       <c r="D16" t="str">
-        <v>2026-05-12</v>
+        <v>2026-05-18</v>
       </c>
       <c r="E16" t="str">
         <v>Shipment</v>
@@ -908,33 +908,33 @@
         <v>Active</v>
       </c>
       <c r="J16" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>BITECOS1358</v>
+        <v>BITECOS1359</v>
       </c>
       <c r="B17" t="str">
-        <v>Sara Connor</v>
+        <v>Ravi Rhanderj</v>
       </c>
       <c r="C17" t="str">
-        <v>sara.connor@gmail.com</v>
+        <v>zensar.demo@brilyant.com</v>
       </c>
       <c r="D17" t="str">
-        <v>2026-05-14</v>
+        <v>2026-05-12</v>
       </c>
       <c r="E17" t="str">
-        <v>Sales</v>
+        <v>Shipment</v>
       </c>
       <c r="F17" t="str">
-        <v>Key Account Manager</v>
+        <v>Python Developer</v>
       </c>
       <c r="G17" t="str">
-        <v>Devakumar N</v>
+        <v>Bhanu Prakash</v>
       </c>
       <c r="H17" t="str">
-        <v xml:space="preserve">HAL Bangalore </v>
+        <v>Coimbatore</v>
       </c>
       <c r="I17" t="str">
         <v>Active</v>
@@ -945,28 +945,28 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>BITECOS1357</v>
+        <v>BITECOS1358</v>
       </c>
       <c r="B18" t="str">
-        <v>Mike Wilson</v>
+        <v>Sara Connor</v>
       </c>
       <c r="C18" t="str">
-        <v>mike.wilson@gmail.com</v>
+        <v>sara.connor@gmail.com</v>
       </c>
       <c r="D18" t="str">
-        <v>2026-05-11</v>
+        <v>2026-05-14</v>
       </c>
       <c r="E18" t="str">
-        <v>Shipment</v>
+        <v>Sales</v>
       </c>
       <c r="F18" t="str">
-        <v>Python Developer</v>
+        <v>Key Account Manager</v>
       </c>
       <c r="G18" t="str">
-        <v>VijayKumar S Kale</v>
+        <v>Devakumar N</v>
       </c>
       <c r="H18" t="str">
-        <v>Coimbatore</v>
+        <v xml:space="preserve">HAL Bangalore </v>
       </c>
       <c r="I18" t="str">
         <v>Active</v>
@@ -977,31 +977,31 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>BITECOS1356</v>
+        <v>BITECOS1357</v>
       </c>
       <c r="B19" t="str">
-        <v>New Intern Employee</v>
+        <v>Mike Wilson</v>
       </c>
       <c r="C19" t="str">
-        <v>test@gmail.com</v>
+        <v>mike.wilson@gmail.com</v>
       </c>
       <c r="D19" t="str">
-        <v>2026-04-09</v>
+        <v>2026-05-11</v>
       </c>
       <c r="E19" t="str">
-        <v>UC</v>
+        <v>Shipment</v>
       </c>
       <c r="F19" t="str">
-        <v>Sr Engineer – AV</v>
+        <v>Python Developer</v>
       </c>
       <c r="G19" t="str">
-        <v>Dinesh Doddaga</v>
+        <v>VijayKumar S Kale</v>
       </c>
       <c r="H19" t="str">
-        <v xml:space="preserve">HAL Bangalore </v>
+        <v>Coimbatore</v>
       </c>
       <c r="I19" t="str">
-        <v>Inactive</v>
+        <v>Active</v>
       </c>
       <c r="J19" t="str">
         <v>Yes</v>
@@ -1009,13 +1009,13 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>BITECOS1355</v>
+        <v>BITECOS1356</v>
       </c>
       <c r="B20" t="str">
-        <v>Swamy Krishna</v>
+        <v>New Intern Employee</v>
       </c>
       <c r="C20" t="str">
-        <v>swamy@yopmail.com</v>
+        <v>test@gmail.com</v>
       </c>
       <c r="D20" t="str">
         <v>2026-04-09</v>
@@ -1027,27 +1027,27 @@
         <v>Sr Engineer – AV</v>
       </c>
       <c r="G20" t="str">
-        <v>Bhanu Prakash</v>
+        <v>Dinesh Doddaga</v>
       </c>
       <c r="H20" t="str">
-        <v>Kerala</v>
+        <v xml:space="preserve">HAL Bangalore </v>
       </c>
       <c r="I20" t="str">
-        <v>Inactive</v>
+        <v>Active</v>
       </c>
       <c r="J20" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>BITECOS1354</v>
+        <v>BITECOS1355</v>
       </c>
       <c r="B21" t="str">
-        <v>Lasya</v>
+        <v>Swamy Krishna</v>
       </c>
       <c r="C21" t="str">
-        <v>lasya.p@brilyant.com</v>
+        <v>swamy@yopmail.com</v>
       </c>
       <c r="D21" t="str">
         <v>2026-04-09</v>
@@ -1059,13 +1059,13 @@
         <v>Sr Engineer – AV</v>
       </c>
       <c r="G21" t="str">
-        <v>Syed khaja Irfanuddin</v>
+        <v>Bhanu Prakash</v>
       </c>
       <c r="H21" t="str">
-        <v>Mumbai</v>
+        <v>Kerala</v>
       </c>
       <c r="I21" t="str">
-        <v>Inactive</v>
+        <v>Active</v>
       </c>
       <c r="J21" t="str">
         <v>No</v>
@@ -1073,28 +1073,28 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>BITECOS1353</v>
+        <v>BITECOS1354</v>
       </c>
       <c r="B22" t="str">
-        <v>Bhanu Prakash</v>
+        <v>Lasya</v>
       </c>
       <c r="C22" t="str">
-        <v>bhanuprakash.r@brilyant.com</v>
+        <v>lasya.p@brilyant.com</v>
       </c>
       <c r="D22" t="str">
-        <v>2021-01-13</v>
+        <v>2026-04-09</v>
       </c>
       <c r="E22" t="str">
-        <v>Finance</v>
+        <v>UC</v>
       </c>
       <c r="F22" t="str">
-        <v>Finance Controller</v>
+        <v>Sr Engineer – AV</v>
       </c>
       <c r="G22" t="str">
-        <v/>
+        <v>Syed khaja Irfanuddin</v>
       </c>
       <c r="H22" t="str">
-        <v>Kozhikode</v>
+        <v>Mumbai</v>
       </c>
       <c r="I22" t="str">
         <v>Active</v>
@@ -1105,28 +1105,28 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>BITECOS1352</v>
+        <v>BITECOS1353</v>
       </c>
       <c r="B23" t="str">
-        <v>Ayushri</v>
+        <v>Bhanu Prakash</v>
       </c>
       <c r="C23" t="str">
-        <v>ayushri.k@brilyant.com</v>
+        <v>bhanuprakash.r@brilyant.com</v>
       </c>
       <c r="D23" t="str">
-        <v>2026-04-01</v>
+        <v>2021-01-13</v>
       </c>
       <c r="E23" t="str">
-        <v>UC</v>
+        <v>Finance</v>
       </c>
       <c r="F23" t="str">
-        <v>Support Engineer - AVSI</v>
+        <v>Finance Controller</v>
       </c>
       <c r="G23" t="str">
-        <v>Syed khaja Irfanuddin</v>
+        <v/>
       </c>
       <c r="H23" t="str">
-        <v>Mumbai</v>
+        <v>Kozhikode</v>
       </c>
       <c r="I23" t="str">
         <v>Active</v>
@@ -1137,28 +1137,28 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>BITECOS1351</v>
+        <v>BITECOS1352</v>
       </c>
       <c r="B24" t="str">
-        <v>S Jagadesh</v>
+        <v>Ayushri</v>
       </c>
       <c r="C24" t="str">
-        <v>jagadesh.s@brilyant.com</v>
+        <v>ayushri.k@brilyant.com</v>
       </c>
       <c r="D24" t="str">
-        <v>2023-02-09</v>
+        <v>2026-04-01</v>
       </c>
       <c r="E24" t="str">
-        <v>Shipment</v>
+        <v>UC</v>
       </c>
       <c r="F24" t="str">
-        <v>Director-Products &amp; SW Development</v>
+        <v>Support Engineer - AVSI</v>
       </c>
       <c r="G24" t="str">
-        <v>Kavya TN</v>
+        <v>Syed khaja Irfanuddin</v>
       </c>
       <c r="H24" t="str">
-        <v>Bangalore</v>
+        <v>Mumbai</v>
       </c>
       <c r="I24" t="str">
         <v>Active</v>
@@ -1169,25 +1169,25 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>BITECOS1350</v>
+        <v>BITECOS1351</v>
       </c>
       <c r="B25" t="str">
-        <v>Sangili Boopathi</v>
+        <v>S Jagadesh</v>
       </c>
       <c r="C25" t="str">
-        <v>sangili.boopathi@brilyant.com</v>
+        <v>jagadesh.s@brilyant.com</v>
       </c>
       <c r="D25" t="str">
-        <v>2026-03-17</v>
+        <v>2023-02-09</v>
       </c>
       <c r="E25" t="str">
-        <v>Finance</v>
+        <v>Shipment</v>
       </c>
       <c r="F25" t="str">
-        <v>Finance Manager</v>
+        <v>Director-Products &amp; SW Development</v>
       </c>
       <c r="G25" t="str">
-        <v>VijayKumar S Kale</v>
+        <v>Kavya TN</v>
       </c>
       <c r="H25" t="str">
         <v>Bangalore</v>
@@ -1201,28 +1201,28 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>BITECOS1349</v>
+        <v>BITECOS1350</v>
       </c>
       <c r="B26" t="str">
-        <v>Kruthi Kumari</v>
+        <v>Sangili Boopathi</v>
       </c>
       <c r="C26" t="str">
-        <v>Kruthi.s@brilynat.com</v>
+        <v>sangili.boopathi@brilyant.com</v>
       </c>
       <c r="D26" t="str">
-        <v>2026-03-10</v>
+        <v>2026-03-17</v>
       </c>
       <c r="E26" t="str">
-        <v>Services</v>
+        <v>Finance</v>
       </c>
       <c r="F26" t="str">
-        <v>Engineering Manager</v>
+        <v>Finance Manager</v>
       </c>
       <c r="G26" t="str">
-        <v>Syed khaja Irfanuddin</v>
+        <v>VijayKumar S Kale</v>
       </c>
       <c r="H26" t="str">
-        <v>Port Blair</v>
+        <v>Bangalore</v>
       </c>
       <c r="I26" t="str">
         <v>Active</v>
@@ -1233,28 +1233,28 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>BITECOS1348</v>
+        <v>BITECOS1349</v>
       </c>
       <c r="B27" t="str">
-        <v>Vulapu Chandrika</v>
+        <v>Kruthi Kumari</v>
       </c>
       <c r="C27" t="str">
-        <v>chandrika.v@brilyant.com</v>
+        <v>Kruthi.s@brilynat.com</v>
       </c>
       <c r="D27" t="str">
-        <v>2026-01-05</v>
+        <v>2026-03-10</v>
       </c>
       <c r="E27" t="str">
-        <v>Finance</v>
+        <v>Services</v>
       </c>
       <c r="F27" t="str">
-        <v>Senior FP&amp;A Analyst</v>
+        <v>Engineering Manager</v>
       </c>
       <c r="G27" t="str">
-        <v>VijayKumar S Kale</v>
+        <v>Syed khaja Irfanuddin</v>
       </c>
       <c r="H27" t="str">
-        <v>Tumkur</v>
+        <v>Port Blair</v>
       </c>
       <c r="I27" t="str">
         <v>Active</v>
@@ -1265,31 +1265,31 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>BITECOS1347</v>
+        <v>BITECOS1348</v>
       </c>
       <c r="B28" t="str">
-        <v>Test Email</v>
+        <v>Vulapu Chandrika</v>
       </c>
       <c r="C28" t="str">
-        <v>test.email@brilyant.com</v>
+        <v>chandrika.v@brilyant.com</v>
       </c>
       <c r="D28" t="str">
-        <v>2025-01-20</v>
+        <v>2026-01-05</v>
       </c>
       <c r="E28" t="str">
-        <v>Shipment</v>
+        <v>Finance</v>
       </c>
       <c r="F28" t="str">
-        <v>Engineering Manager</v>
+        <v>Senior FP&amp;A Analyst</v>
       </c>
       <c r="G28" t="str">
-        <v>Devakumar N</v>
+        <v>VijayKumar S Kale</v>
       </c>
       <c r="H28" t="str">
-        <v>Bangalore</v>
+        <v>Tumkur</v>
       </c>
       <c r="I28" t="str">
-        <v>Inactive</v>
+        <v>Active</v>
       </c>
       <c r="J28" t="str">
         <v>No</v>
@@ -1297,28 +1297,28 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>BITECOS1346</v>
+        <v>BITECOS1347</v>
       </c>
       <c r="B29" t="str">
-        <v>Kavya TN</v>
+        <v>Test Email</v>
       </c>
       <c r="C29" t="str">
-        <v>kavya.tn@brilyant.com</v>
+        <v>test.email@brilyant.com</v>
       </c>
       <c r="D29" t="str">
-        <v>2020-03-10</v>
+        <v>2025-01-20</v>
       </c>
       <c r="E29" t="str">
-        <v>Finance</v>
+        <v>Shipment</v>
       </c>
       <c r="F29" t="str">
-        <v>Senior FP&amp;A Analyst</v>
+        <v>Engineering Manager</v>
       </c>
       <c r="G29" t="str">
-        <v>Bhanu Prakash</v>
+        <v>Devakumar N</v>
       </c>
       <c r="H29" t="str">
-        <v>Kerala</v>
+        <v>Bangalore</v>
       </c>
       <c r="I29" t="str">
         <v>Active</v>
@@ -1329,28 +1329,28 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>BITECOS1345</v>
+        <v>BITECOS1346</v>
       </c>
       <c r="B30" t="str">
-        <v>Rajendra singh</v>
+        <v>Kavya TN</v>
       </c>
       <c r="C30" t="str">
-        <v>Rajendra.singh@brilyant.com</v>
+        <v>kavya.tn@brilyant.com</v>
       </c>
       <c r="D30" t="str">
-        <v>2022-12-07</v>
+        <v>2020-03-10</v>
       </c>
       <c r="E30" t="str">
-        <v>Networking</v>
+        <v>Finance</v>
       </c>
       <c r="F30" t="str">
-        <v>Business Development Manager- Networking</v>
+        <v>Senior FP&amp;A Analyst</v>
       </c>
       <c r="G30" t="str">
-        <v>Sagarika</v>
+        <v>Bhanu Prakash</v>
       </c>
       <c r="H30" t="str">
-        <v>Bangalore</v>
+        <v>Kerala</v>
       </c>
       <c r="I30" t="str">
         <v>Active</v>
@@ -1361,25 +1361,25 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>BITECOS1344</v>
+        <v>BITECOS1345</v>
       </c>
       <c r="B31" t="str">
-        <v>Ganesh Mali</v>
+        <v>Rajendra singh</v>
       </c>
       <c r="C31" t="str">
-        <v>ganesh.mali@brilyant.com</v>
+        <v>Rajendra.singh@brilyant.com</v>
       </c>
       <c r="D31" t="str">
-        <v>2024-03-10</v>
+        <v>2022-12-07</v>
       </c>
       <c r="E31" t="str">
-        <v>Shipment</v>
+        <v>Networking</v>
       </c>
       <c r="F31" t="str">
-        <v>Engineering Manager</v>
+        <v>Business Development Manager- Networking</v>
       </c>
       <c r="G31" t="str">
-        <v>Devakumar N</v>
+        <v>Sagarika</v>
       </c>
       <c r="H31" t="str">
         <v>Bangalore</v>
@@ -1393,31 +1393,31 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>BITECOS1343</v>
+        <v>BITECOS1344</v>
       </c>
       <c r="B32" t="str">
-        <v xml:space="preserve">Test Attendance 2 </v>
+        <v>Ganesh Mali</v>
       </c>
       <c r="C32" t="str">
-        <v>testattandance2@yopmail.com</v>
+        <v>ganesh.mali@brilyant.com</v>
       </c>
       <c r="D32" t="str">
-        <v>2026-02-01</v>
+        <v>2024-03-10</v>
       </c>
       <c r="E32" t="str">
-        <v>Quality Assurance (QA)</v>
+        <v>Shipment</v>
       </c>
       <c r="F32" t="str">
-        <v>Quality Associate Analyst</v>
+        <v>Engineering Manager</v>
       </c>
       <c r="G32" t="str">
-        <v>Rajendra singh</v>
+        <v>Devakumar N</v>
       </c>
       <c r="H32" t="str">
         <v>Bangalore</v>
       </c>
       <c r="I32" t="str">
-        <v>Inactive</v>
+        <v>Active</v>
       </c>
       <c r="J32" t="str">
         <v>No</v>
@@ -1425,13 +1425,13 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>BITECOS1342</v>
+        <v>BITECOS1343</v>
       </c>
       <c r="B33" t="str">
-        <v>Test Attandance 1</v>
+        <v xml:space="preserve">Test Attendance 2 </v>
       </c>
       <c r="C33" t="str">
-        <v>attandance1@yopmail.com</v>
+        <v>testattandance2@yopmail.com</v>
       </c>
       <c r="D33" t="str">
         <v>2026-02-01</v>
@@ -1446,10 +1446,10 @@
         <v>Rajendra singh</v>
       </c>
       <c r="H33" t="str">
-        <v>Tumkur</v>
+        <v>Bangalore</v>
       </c>
       <c r="I33" t="str">
-        <v>Inactive</v>
+        <v>Active</v>
       </c>
       <c r="J33" t="str">
         <v>No</v>
@@ -1457,31 +1457,31 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>BITECOS1341</v>
+        <v>BITECOS1342</v>
       </c>
       <c r="B34" t="str">
-        <v>testing email</v>
+        <v>Test Attandance 1</v>
       </c>
       <c r="C34" t="str">
-        <v>emailtesting12345@yopmail.com</v>
+        <v>attandance1@yopmail.com</v>
       </c>
       <c r="D34" t="str">
-        <v>2025-10-20</v>
+        <v>2026-02-01</v>
       </c>
       <c r="E34" t="str">
-        <v>UC</v>
+        <v>Quality Assurance (QA)</v>
       </c>
       <c r="F34" t="str">
-        <v>Senior Support Specialist - UC</v>
+        <v>Quality Associate Analyst</v>
       </c>
       <c r="G34" t="str">
-        <v>Bandi Prasanth Babu</v>
+        <v>Rajendra singh</v>
       </c>
       <c r="H34" t="str">
         <v>Tumkur</v>
       </c>
       <c r="I34" t="str">
-        <v>Inactive</v>
+        <v>Active</v>
       </c>
       <c r="J34" t="str">
         <v>No</v>
@@ -1489,31 +1489,31 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>BITECOS1340</v>
+        <v>BITECOS1341</v>
       </c>
       <c r="B35" t="str">
-        <v>New CC</v>
+        <v>testing email</v>
       </c>
       <c r="C35" t="str">
-        <v>new-cc@brilyant.com</v>
+        <v>emailtesting12345@yopmail.com</v>
       </c>
       <c r="D35" t="str">
-        <v>2025-09-22</v>
+        <v>2025-10-20</v>
       </c>
       <c r="E35" t="str">
-        <v>Quality Assurance (QA)</v>
+        <v>UC</v>
       </c>
       <c r="F35" t="str">
-        <v>QA Engineer</v>
+        <v>Senior Support Specialist - UC</v>
       </c>
       <c r="G35" t="str">
         <v>Bandi Prasanth Babu</v>
       </c>
       <c r="H35" t="str">
-        <v>Bangalore</v>
+        <v>Tumkur</v>
       </c>
       <c r="I35" t="str">
-        <v>Inactive</v>
+        <v>Active</v>
       </c>
       <c r="J35" t="str">
         <v>No</v>
@@ -1521,28 +1521,28 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>BITECOS1339</v>
+        <v>BITECOS1340</v>
       </c>
       <c r="B36" t="str">
-        <v xml:space="preserve"> Selvaganapathi K</v>
+        <v>New CC</v>
       </c>
       <c r="C36" t="str">
-        <v>selvaganapathi.k@brilyant.com</v>
+        <v>new-cc@brilyant.com</v>
       </c>
       <c r="D36" t="str">
-        <v>2023-02-07</v>
+        <v>2025-09-22</v>
       </c>
       <c r="E36" t="str">
-        <v>Networking</v>
+        <v>Quality Assurance (QA)</v>
       </c>
       <c r="F36" t="str">
-        <v>Presales Specialist- AVSI</v>
+        <v>QA Engineer</v>
       </c>
       <c r="G36" t="str">
-        <v>Rajendra singh</v>
+        <v>Bandi Prasanth Babu</v>
       </c>
       <c r="H36" t="str">
-        <v>Mumbai</v>
+        <v>Bangalore</v>
       </c>
       <c r="I36" t="str">
         <v>Active</v>
@@ -1553,28 +1553,28 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>BITECOS1338</v>
+        <v>BITECOS1339</v>
       </c>
       <c r="B37" t="str">
-        <v>Dinesh Doddaga</v>
+        <v xml:space="preserve"> Selvaganapathi K</v>
       </c>
       <c r="C37" t="str">
-        <v>dinesh.doddaga@brilyant.com</v>
+        <v>selvaganapathi.k@brilyant.com</v>
       </c>
       <c r="D37" t="str">
-        <v>2025-03-10</v>
+        <v>2023-02-07</v>
       </c>
       <c r="E37" t="str">
-        <v>Logistics</v>
+        <v>Networking</v>
       </c>
       <c r="F37" t="str">
-        <v>Admin Manager</v>
+        <v>Presales Specialist- AVSI</v>
       </c>
       <c r="G37" t="str">
-        <v>Syed khaja Irfanuddin</v>
+        <v>Rajendra singh</v>
       </c>
       <c r="H37" t="str">
-        <v>Kozhikode</v>
+        <v>Mumbai</v>
       </c>
       <c r="I37" t="str">
         <v>Active</v>
@@ -1585,28 +1585,28 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>BITECOS1337</v>
+        <v>BITECOS1338</v>
       </c>
       <c r="B38" t="str">
-        <v>Mohanpradeep V</v>
+        <v>Dinesh Doddaga</v>
       </c>
       <c r="C38" t="str">
-        <v>mohanpradeep.v@brilyant.com</v>
+        <v>dinesh.doddaga@brilyant.com</v>
       </c>
       <c r="D38" t="str">
-        <v>2021-03-10</v>
+        <v>2025-03-10</v>
       </c>
       <c r="E38" t="str">
-        <v>Networking</v>
+        <v>Logistics</v>
       </c>
       <c r="F38" t="str">
-        <v>Cyber Security Analyst</v>
+        <v>Admin Manager</v>
       </c>
       <c r="G38" t="str">
-        <v>Rajendra singh</v>
+        <v>Syed khaja Irfanuddin</v>
       </c>
       <c r="H38" t="str">
-        <v>Mumbai</v>
+        <v>Kozhikode</v>
       </c>
       <c r="I38" t="str">
         <v>Active</v>
@@ -1617,28 +1617,28 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>BITECOS1335</v>
+        <v>BITECOS1337</v>
       </c>
       <c r="B39" t="str">
-        <v>Venkateswarlu</v>
+        <v>Mohanpradeep V</v>
       </c>
       <c r="C39" t="str">
-        <v>venkateswarlu.v@brilyant.com</v>
+        <v>mohanpradeep.v@brilyant.com</v>
       </c>
       <c r="D39" t="str">
-        <v>2016-03-10</v>
+        <v>2021-03-10</v>
       </c>
       <c r="E39" t="str">
         <v>Networking</v>
       </c>
       <c r="F39" t="str">
-        <v>Support Engineer</v>
+        <v>Cyber Security Analyst</v>
       </c>
       <c r="G39" t="str">
         <v>Rajendra singh</v>
       </c>
       <c r="H39" t="str">
-        <v>Kozhikode</v>
+        <v>Mumbai</v>
       </c>
       <c r="I39" t="str">
         <v>Active</v>
@@ -1649,28 +1649,28 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>BITECOS1334</v>
+        <v>BITECOS1335</v>
       </c>
       <c r="B40" t="str">
-        <v xml:space="preserve">Pendem Nethri </v>
+        <v>Venkateswarlu</v>
       </c>
       <c r="C40" t="str">
-        <v>nethri.t@brilyant.com</v>
+        <v>venkateswarlu.v@brilyant.com</v>
       </c>
       <c r="D40" t="str">
-        <v>2024-01-08</v>
+        <v>2016-03-10</v>
       </c>
       <c r="E40" t="str">
-        <v>Shipment</v>
+        <v>Networking</v>
       </c>
       <c r="F40" t="str">
-        <v>Customer  Executive</v>
+        <v>Support Engineer</v>
       </c>
       <c r="G40" t="str">
-        <v>Harsh Kumar</v>
+        <v>Rajendra singh</v>
       </c>
       <c r="H40" t="str">
-        <v>andaman and nicobar islands</v>
+        <v>Kozhikode</v>
       </c>
       <c r="I40" t="str">
         <v>Active</v>
@@ -1681,28 +1681,28 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>BITECOS1333</v>
+        <v>BITECOS1334</v>
       </c>
       <c r="B41" t="str">
-        <v>Sagarika</v>
+        <v xml:space="preserve">Pendem Nethri </v>
       </c>
       <c r="C41" t="str">
-        <v>sagarika@brilyant.com</v>
+        <v>nethri.t@brilyant.com</v>
       </c>
       <c r="D41" t="str">
-        <v>2024-01-05</v>
+        <v>2024-01-08</v>
       </c>
       <c r="E41" t="str">
-        <v>Networking</v>
+        <v>Shipment</v>
       </c>
       <c r="F41" t="str">
-        <v>Presales Consultant – Enterprise</v>
+        <v>Customer  Executive</v>
       </c>
       <c r="G41" t="str">
-        <v>S Jagadesh</v>
+        <v>Harsh Kumar</v>
       </c>
       <c r="H41" t="str">
-        <v>Port Blair</v>
+        <v>andaman and nicobar islands</v>
       </c>
       <c r="I41" t="str">
         <v>Active</v>
@@ -1713,28 +1713,28 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>BITECOS1332</v>
+        <v>BITECOS1333</v>
       </c>
       <c r="B42" t="str">
-        <v>Harsh Kumar</v>
+        <v>Sagarika</v>
       </c>
       <c r="C42" t="str">
-        <v>harsh.kumar@brilyant.com</v>
+        <v>sagarika@brilyant.com</v>
       </c>
       <c r="D42" t="str">
-        <v>2011-03-10</v>
+        <v>2024-01-05</v>
       </c>
       <c r="E42" t="str">
-        <v>Shipment</v>
+        <v>Networking</v>
       </c>
       <c r="F42" t="str">
-        <v>BDM- Enterprise Infra Solutions</v>
+        <v>Presales Consultant – Enterprise</v>
       </c>
       <c r="G42" t="str">
         <v>S Jagadesh</v>
       </c>
       <c r="H42" t="str">
-        <v xml:space="preserve">HAL Bangalore </v>
+        <v>Port Blair</v>
       </c>
       <c r="I42" t="str">
         <v>Active</v>
@@ -1745,28 +1745,28 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>BITECOS1331</v>
+        <v>BITECOS1332</v>
       </c>
       <c r="B43" t="str">
-        <v>Narimeti Thrisha</v>
+        <v>Harsh Kumar</v>
       </c>
       <c r="C43" t="str">
-        <v>narimeti.thrisha@brilyant.com</v>
+        <v>harsh.kumar@brilyant.com</v>
       </c>
       <c r="D43" t="str">
-        <v>2024-01-05</v>
+        <v>2011-03-10</v>
       </c>
       <c r="E43" t="str">
-        <v>Finance</v>
+        <v>Shipment</v>
       </c>
       <c r="F43" t="str">
-        <v>Senior FP&amp;A Analyst</v>
+        <v>BDM- Enterprise Infra Solutions</v>
       </c>
       <c r="G43" t="str">
-        <v>VijayKumar S Kale</v>
+        <v>S Jagadesh</v>
       </c>
       <c r="H43" t="str">
-        <v>Kerala</v>
+        <v xml:space="preserve">HAL Bangalore </v>
       </c>
       <c r="I43" t="str">
         <v>Active</v>
@@ -1777,28 +1777,28 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>BITECOS1330</v>
+        <v>BITECOS1331</v>
       </c>
       <c r="B44" t="str">
-        <v>Hrassistant</v>
+        <v>Narimeti Thrisha</v>
       </c>
       <c r="C44" t="str">
-        <v>Hrassistant@brilyant.com</v>
+        <v>narimeti.thrisha@brilyant.com</v>
       </c>
       <c r="D44" t="str">
-        <v>2025-06-23</v>
+        <v>2024-01-05</v>
       </c>
       <c r="E44" t="str">
-        <v>Administration</v>
+        <v>Finance</v>
       </c>
       <c r="F44" t="str">
-        <v>Quality Associate Analyst</v>
+        <v>Senior FP&amp;A Analyst</v>
       </c>
       <c r="G44" t="str">
-        <v>Bhanu Prakash</v>
+        <v>VijayKumar S Kale</v>
       </c>
       <c r="H44" t="str">
-        <v xml:space="preserve">HAL Bangalore </v>
+        <v>Kerala</v>
       </c>
       <c r="I44" t="str">
         <v>Active</v>
@@ -1809,28 +1809,28 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>BITECOS1329</v>
+        <v>BITECOS1330</v>
       </c>
       <c r="B45" t="str">
-        <v>Manya</v>
+        <v>Hrassistant</v>
       </c>
       <c r="C45" t="str">
-        <v>manyatha@yopmail.com</v>
+        <v>Hrassistant@brilyant.com</v>
       </c>
       <c r="D45" t="str">
-        <v>2023-01-09</v>
+        <v>2025-06-23</v>
       </c>
       <c r="E45" t="str">
-        <v>Shipment</v>
+        <v>Administration</v>
       </c>
       <c r="F45" t="str">
-        <v>Sr Engineer – AV</v>
+        <v>Quality Associate Analyst</v>
       </c>
       <c r="G45" t="str">
-        <v>Devakumar N</v>
+        <v>Bhanu Prakash</v>
       </c>
       <c r="H45" t="str">
-        <v>Gurugram</v>
+        <v xml:space="preserve">HAL Bangalore </v>
       </c>
       <c r="I45" t="str">
         <v>Active</v>
@@ -1841,28 +1841,28 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>BITECOS1328</v>
+        <v>BITECOS1329</v>
       </c>
       <c r="B46" t="str">
-        <v>Khushi Shetty</v>
+        <v>Manya</v>
       </c>
       <c r="C46" t="str">
-        <v>khushishetty@yopmail.com</v>
+        <v>manyatha@yopmail.com</v>
       </c>
       <c r="D46" t="str">
-        <v>2023-01-02</v>
+        <v>2023-01-09</v>
       </c>
       <c r="E46" t="str">
         <v>Shipment</v>
       </c>
       <c r="F46" t="str">
-        <v>Senior Support Specialist - UC</v>
+        <v>Sr Engineer – AV</v>
       </c>
       <c r="G46" t="str">
         <v>Devakumar N</v>
       </c>
       <c r="H46" t="str">
-        <v>andaman and nicobar islands</v>
+        <v>Gurugram</v>
       </c>
       <c r="I46" t="str">
         <v>Active</v>
@@ -1873,28 +1873,28 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>BITECOS1288</v>
+        <v>BITECOS1328</v>
       </c>
       <c r="B47" t="str">
-        <v>Suman Mahendrakar</v>
+        <v>Khushi Shetty</v>
       </c>
       <c r="C47" t="str">
-        <v>suman.k@brilyant.com</v>
+        <v>khushishetty@yopmail.com</v>
       </c>
       <c r="D47" t="str">
-        <v>2014-06-09</v>
+        <v>2023-01-02</v>
       </c>
       <c r="E47" t="str">
-        <v>Logistics</v>
+        <v>Shipment</v>
       </c>
       <c r="F47" t="str">
-        <v>QA Engineer</v>
+        <v>Senior Support Specialist - UC</v>
       </c>
       <c r="G47" t="str">
-        <v>Bandi Prasanth Babu</v>
+        <v>Devakumar N</v>
       </c>
       <c r="H47" t="str">
-        <v>Bangalore</v>
+        <v>andaman and nicobar islands</v>
       </c>
       <c r="I47" t="str">
         <v>Active</v>
@@ -1905,25 +1905,25 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>BITECOS1327</v>
+        <v>BITECOS1288</v>
       </c>
       <c r="B48" t="str">
-        <v>Bandi Prasanth Babu</v>
+        <v>Suman Mahendrakar</v>
       </c>
       <c r="C48" t="str">
-        <v>prasanth.babu@brilyant.com</v>
+        <v>suman.k@brilyant.com</v>
       </c>
       <c r="D48" t="str">
-        <v>2025-07-21</v>
+        <v>2014-06-09</v>
       </c>
       <c r="E48" t="str">
         <v>Logistics</v>
       </c>
       <c r="F48" t="str">
-        <v>Engineering Manager</v>
+        <v>QA Engineer</v>
       </c>
       <c r="G48" t="str">
-        <v>Dinesh Doddaga</v>
+        <v>Bandi Prasanth Babu</v>
       </c>
       <c r="H48" t="str">
         <v>Bangalore</v>
@@ -1937,25 +1937,25 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>BITECOS1234</v>
+        <v>BITECOS1327</v>
       </c>
       <c r="B49" t="str">
-        <v>Disha S. Bagewadi</v>
+        <v>Bandi Prasanth Babu</v>
       </c>
       <c r="C49" t="str">
-        <v>disha.s@brilyant.com</v>
+        <v>prasanth.babu@brilyant.com</v>
       </c>
       <c r="D49" t="str">
-        <v>2025-01-06</v>
+        <v>2025-07-21</v>
       </c>
       <c r="E49" t="str">
         <v>Logistics</v>
       </c>
       <c r="F49" t="str">
-        <v>Trainee - Software Development</v>
+        <v>Engineering Manager</v>
       </c>
       <c r="G49" t="str">
-        <v>Bandi Prasanth Babu</v>
+        <v>Dinesh Doddaga</v>
       </c>
       <c r="H49" t="str">
         <v>Bangalore</v>
@@ -1969,28 +1969,28 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>BITECOS1326</v>
+        <v>BITECOS1234</v>
       </c>
       <c r="B50" t="str">
-        <v>Gattu Ashwitha</v>
+        <v>Disha S. Bagewadi</v>
       </c>
       <c r="C50" t="str">
-        <v>gattu.ashwitha@brilyant.com</v>
+        <v>disha.s@brilyant.com</v>
       </c>
       <c r="D50" t="str">
-        <v>2024-10-22</v>
+        <v>2025-01-06</v>
       </c>
       <c r="E50" t="str">
-        <v>Finance</v>
+        <v>Logistics</v>
       </c>
       <c r="F50" t="str">
-        <v>Senior FP&amp;A Analyst</v>
+        <v>Trainee - Software Development</v>
       </c>
       <c r="G50" t="str">
-        <v>Kavya TN</v>
+        <v>Bandi Prasanth Babu</v>
       </c>
       <c r="H50" t="str">
-        <v>Mumbai</v>
+        <v>Bangalore</v>
       </c>
       <c r="I50" t="str">
         <v>Active</v>
@@ -2001,16 +2001,16 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>BITECOS1214</v>
+        <v>BITECOS1326</v>
       </c>
       <c r="B51" t="str">
-        <v>VijayKumar S Kale</v>
+        <v>Gattu Ashwitha</v>
       </c>
       <c r="C51" t="str">
-        <v>VijayKumar.S@brilyant.com</v>
+        <v>gattu.ashwitha@brilyant.com</v>
       </c>
       <c r="D51" t="str">
-        <v>2024-10-07</v>
+        <v>2024-10-22</v>
       </c>
       <c r="E51" t="str">
         <v>Finance</v>
@@ -2019,10 +2019,10 @@
         <v>Senior FP&amp;A Analyst</v>
       </c>
       <c r="G51" t="str">
-        <v>Gattu Ashwitha</v>
+        <v>Kavya TN</v>
       </c>
       <c r="H51" t="str">
-        <v>Bangalore</v>
+        <v>Mumbai</v>
       </c>
       <c r="I51" t="str">
         <v>Active</v>
@@ -2033,25 +2033,25 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>BITECOS1121</v>
+        <v>BITECOS1214</v>
       </c>
       <c r="B52" t="str">
-        <v>Syed khaja Irfanuddin</v>
+        <v>VijayKumar S Kale</v>
       </c>
       <c r="C52" t="str">
-        <v>Syed.Irfanuddin@brilyant.com</v>
+        <v>VijayKumar.S@brilyant.com</v>
       </c>
       <c r="D52" t="str">
-        <v>2023-08-07</v>
+        <v>2024-10-07</v>
       </c>
       <c r="E52" t="str">
-        <v>Logistics</v>
+        <v>Finance</v>
       </c>
       <c r="F52" t="str">
-        <v>Director-Products &amp; SW Development</v>
+        <v>Senior FP&amp;A Analyst</v>
       </c>
       <c r="G52" t="str">
-        <v>S Jagadesh</v>
+        <v>Gattu Ashwitha</v>
       </c>
       <c r="H52" t="str">
         <v>Bangalore</v>
@@ -2065,25 +2065,25 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>BITECOS1141</v>
+        <v>BITECOS1121</v>
       </c>
       <c r="B53" t="str">
-        <v>Devakumar N</v>
+        <v>Syed khaja Irfanuddin</v>
       </c>
       <c r="C53" t="str">
-        <v>devakumar@brilyant.com</v>
+        <v>Syed.Irfanuddin@brilyant.com</v>
       </c>
       <c r="D53" t="str">
-        <v>2023-12-07</v>
+        <v>2023-08-07</v>
       </c>
       <c r="E53" t="str">
-        <v>Shipment</v>
+        <v>Logistics</v>
       </c>
       <c r="F53" t="str">
-        <v>Software Developer</v>
+        <v>Director-Products &amp; SW Development</v>
       </c>
       <c r="G53" t="str">
-        <v xml:space="preserve">Pendem Nethri </v>
+        <v>S Jagadesh</v>
       </c>
       <c r="H53" t="str">
         <v>Bangalore</v>
@@ -2097,25 +2097,25 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>BITECOS1137</v>
+        <v>BITECOS1141</v>
       </c>
       <c r="B54" t="str">
-        <v>Ramesh Mali</v>
+        <v>Devakumar N</v>
       </c>
       <c r="C54" t="str">
-        <v>Ramesh.mali@brilyant.com</v>
+        <v>devakumar@brilyant.com</v>
       </c>
       <c r="D54" t="str">
-        <v>2023-03-23</v>
+        <v>2023-12-07</v>
       </c>
       <c r="E54" t="str">
-        <v>UC</v>
+        <v>Shipment</v>
       </c>
       <c r="F54" t="str">
-        <v>Lead Developer</v>
+        <v>Software Developer</v>
       </c>
       <c r="G54" t="str">
-        <v>Ayushri</v>
+        <v xml:space="preserve">Pendem Nethri </v>
       </c>
       <c r="H54" t="str">
         <v>Bangalore</v>
@@ -2127,9 +2127,41 @@
         <v>No</v>
       </c>
     </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>BITECOS1137</v>
+      </c>
+      <c r="B55" t="str">
+        <v>Ramesh Mali</v>
+      </c>
+      <c r="C55" t="str">
+        <v>Ramesh.mali@brilyant.com</v>
+      </c>
+      <c r="D55" t="str">
+        <v>2023-03-23</v>
+      </c>
+      <c r="E55" t="str">
+        <v>UC</v>
+      </c>
+      <c r="F55" t="str">
+        <v>Lead Developer</v>
+      </c>
+      <c r="G55" t="str">
+        <v>Ayushri</v>
+      </c>
+      <c r="H55" t="str">
+        <v>Bangalore</v>
+      </c>
+      <c r="I55" t="str">
+        <v>Active</v>
+      </c>
+      <c r="J55" t="str">
+        <v>No</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J54"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J55"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>